<commit_message>
#16 Client and eSpark BOM Updated.
</commit_message>
<xml_diff>
--- a/Design-Files/OFP_VIM_v1.5/BOM/Client-BOM-OFP_VIM_v1.5.xlsx
+++ b/Design-Files/OFP_VIM_v1.5/BOM/Client-BOM-OFP_VIM_v1.5.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView minimized="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="237">
   <si>
     <t>#</t>
   </si>
@@ -162,9 +162,6 @@
     <t>L1, L2, L3, L5, L6, L7</t>
   </si>
   <si>
-    <t>L4</t>
-  </si>
-  <si>
     <t>Q1</t>
   </si>
   <si>
@@ -297,12 +294,6 @@
     <t>CONN HDR 24POS 0.1 GOLD PCB R/A</t>
   </si>
   <si>
-    <t>450V 17.5A 4 Bend -40℃~+105℃ 1 5.08mm Green Board Edge/Receptacle-Open Push-Pull,P=5.08mm Pluggable System Terminal Block ROHS</t>
-  </si>
-  <si>
-    <t>450V 17.5A 4 -40℃~+105℃ 1.5 1 14~28 5.08mm 1x4P Green Plug P=5.08mm Pluggable System Terminal Block ROHS</t>
-  </si>
-  <si>
     <t>420mA 470uH EI-core Inductor ±20% Plugin Power Inductors ROHS</t>
   </si>
   <si>
@@ -414,9 +405,6 @@
     <t>SFH11-PBPC-D12-RA-BK</t>
   </si>
   <si>
-    <t>DB2ER-5.08-4P-GN</t>
-  </si>
-  <si>
     <t>PK0810-471MB</t>
   </si>
   <si>
@@ -504,9 +492,6 @@
     <t>BLM21BD152SN1D</t>
   </si>
   <si>
-    <t>DB2EK-5.08-4P-GN-S</t>
-  </si>
-  <si>
     <t>IPD90R1K2C3</t>
   </si>
   <si>
@@ -603,12 +588,6 @@
     <t>Sullins</t>
   </si>
   <si>
-    <t>DIBO</t>
-  </si>
-  <si>
-    <t>DORABO</t>
-  </si>
-  <si>
     <t>SXN(Shun Xiang Nuo Elec)</t>
   </si>
   <si>
@@ -727,6 +706,30 @@
   </si>
   <si>
     <t>Design From Custom Supplier</t>
+  </si>
+  <si>
+    <t>Plugin,P=3.81mm Pluggable System Terminal Block ROHS</t>
+  </si>
+  <si>
+    <t>KF2EDGRG-3.81-4P</t>
+  </si>
+  <si>
+    <t>Cixi Kefa Elec</t>
+  </si>
+  <si>
+    <t>-40℃~+105℃ 1.5 1 16~28 3.81mm 160V 7A 4 1x4P Green Plug Snap Fit P=3.81mm Pluggable System Terminal Block ROHS</t>
+  </si>
+  <si>
+    <t>KF2EDGKNG-3.81-4P</t>
+  </si>
+  <si>
+    <t>T1</t>
+  </si>
+  <si>
+    <t>12V/1.5A transformer</t>
+  </si>
+  <si>
+    <t>FTEFD25-037</t>
   </si>
 </sst>
 </file>
@@ -940,7 +943,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1242,7 +1245,10 @@
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.85546875" customWidth="1"/>
+    <col min="13" max="13" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1270,25 +1276,25 @@
         <v>21</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1304,19 +1310,19 @@
         <v>22</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="J3" s="7">
         <v>2</v>
@@ -1336,19 +1342,19 @@
         <v>23</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="J4" s="9">
         <v>3</v>
@@ -1368,19 +1374,19 @@
         <v>24</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="J5" s="7">
         <v>2</v>
@@ -1400,19 +1406,19 @@
         <v>25</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="J6" s="9">
         <v>4</v>
@@ -1432,19 +1438,19 @@
         <v>26</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="J7" s="7">
         <v>1</v>
@@ -1464,19 +1470,19 @@
         <v>27</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="J8" s="9">
         <v>1</v>
@@ -1496,19 +1502,19 @@
         <v>28</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
@@ -1528,19 +1534,19 @@
         <v>29</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="J10" s="9">
         <v>1</v>
@@ -1560,19 +1566,19 @@
         <v>30</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="J11" s="7">
         <v>1</v>
@@ -1592,19 +1598,19 @@
         <v>31</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="J12" s="9">
         <v>2</v>
@@ -1624,19 +1630,19 @@
         <v>32</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="J13" s="7">
         <v>1</v>
@@ -1656,19 +1662,19 @@
         <v>33</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
@@ -1688,19 +1694,19 @@
         <v>34</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="J15" s="7">
         <v>3</v>
@@ -1720,19 +1726,19 @@
         <v>35</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="J16" s="9">
         <v>6</v>
@@ -1752,19 +1758,19 @@
         <v>36</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="J17" s="7">
         <v>1</v>
@@ -1784,19 +1790,19 @@
         <v>37</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="H18" s="9" t="s">
         <v>7</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="J18" s="9">
         <v>1</v>
@@ -1816,19 +1822,19 @@
         <v>38</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="H19" s="7" t="s">
         <v>7</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="J19" s="7">
         <v>1</v>
@@ -1848,19 +1854,19 @@
         <v>39</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="H20" s="9" t="s">
         <v>7</v>
       </c>
       <c r="I20" s="8" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="J20" s="9">
         <v>1</v>
@@ -1880,19 +1886,19 @@
         <v>40</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="J21" s="7">
         <v>1</v>
@@ -1912,19 +1918,19 @@
         <v>41</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="I22" s="8" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="J22" s="9">
         <v>4</v>
@@ -1944,19 +1950,19 @@
         <v>42</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="J23" s="7">
         <v>1</v>
@@ -1976,26 +1982,26 @@
         <v>43</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="I24" s="8" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="J24" s="9">
         <v>1</v>
       </c>
       <c r="K24" s="9"/>
     </row>
-    <row r="25" spans="1:11" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="11">
         <f>ROW(B25) - ROW($B$2)</f>
@@ -2008,19 +2014,19 @@
         <v>44</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>92</v>
+        <v>229</v>
       </c>
       <c r="F25" s="9" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>131</v>
+        <v>230</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>194</v>
+        <v>231</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="J25" s="7">
         <v>1</v>
@@ -2040,19 +2046,19 @@
         <v>45</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>93</v>
+        <v>232</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>161</v>
+        <v>233</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>195</v>
-      </c>
-      <c r="I26" s="8" t="s">
-        <v>233</v>
+        <v>231</v>
+      </c>
+      <c r="I26" s="10" t="s">
+        <v>226</v>
       </c>
       <c r="J26" s="9">
         <v>1</v>
@@ -2072,120 +2078,120 @@
         <v>46</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="J27" s="7">
         <v>6</v>
       </c>
       <c r="K27" s="7"/>
     </row>
-    <row r="28" spans="1:11" ht="51.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="11">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C28" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="D28" s="9" t="s">
+      <c r="C28" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D28" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="E28" s="10" t="s">
-        <v>233</v>
-      </c>
-      <c r="F28" s="9" t="s">
-        <v>234</v>
-      </c>
-      <c r="G28" s="10" t="s">
-        <v>233</v>
-      </c>
-      <c r="H28" s="9"/>
+      <c r="E28" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="G28" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>190</v>
+      </c>
       <c r="I28" s="10" t="s">
-        <v>233</v>
-      </c>
-      <c r="J28" s="9">
-        <v>1</v>
-      </c>
-      <c r="K28" s="15" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>226</v>
+      </c>
+      <c r="J28" s="7">
+        <v>1</v>
+      </c>
+      <c r="K28" s="7"/>
+    </row>
+    <row r="29" spans="1:11" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="11">
         <f>ROW(B29) - ROW($B$2)</f>
         <v>27</v>
       </c>
-      <c r="C29" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="D29" s="7" t="s">
+      <c r="C29" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="D29" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="E29" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="F29" s="7" t="s">
-        <v>133</v>
-      </c>
-      <c r="G29" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="H29" s="7" t="s">
-        <v>197</v>
+      <c r="E29" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="F29" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="G29" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="H29" s="9" t="s">
+        <v>185</v>
       </c>
       <c r="I29" s="10" t="s">
-        <v>233</v>
-      </c>
-      <c r="J29" s="7">
-        <v>1</v>
-      </c>
-      <c r="K29" s="7"/>
-    </row>
-    <row r="30" spans="1:11" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>208</v>
+      </c>
+      <c r="J29" s="9">
+        <v>3</v>
+      </c>
+      <c r="K29" s="9"/>
+    </row>
+    <row r="30" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="11">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="C30" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="D30" s="9" t="s">
+      <c r="C30" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D30" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="E30" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="F30" s="9" t="s">
-        <v>234</v>
-      </c>
-      <c r="G30" s="10" t="s">
-        <v>134</v>
-      </c>
-      <c r="H30" s="9" t="s">
-        <v>190</v>
-      </c>
-      <c r="I30" s="10" t="s">
-        <v>215</v>
-      </c>
-      <c r="J30" s="9">
-        <v>3</v>
-      </c>
-      <c r="K30" s="9"/>
+      <c r="E30" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="G30" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="H30" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I30" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="J30" s="7">
+        <v>6</v>
+      </c>
+      <c r="K30" s="7"/>
     </row>
     <row r="31" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
@@ -2193,31 +2199,31 @@
         <f>ROW(B31) - ROW($B$2)</f>
         <v>29</v>
       </c>
-      <c r="C31" s="12" t="s">
+      <c r="C31" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="D31" s="7" t="s">
+      <c r="D31" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="E31" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="F31" s="7" t="s">
-        <v>135</v>
-      </c>
-      <c r="G31" s="8" t="s">
-        <v>163</v>
-      </c>
-      <c r="H31" s="7" t="s">
-        <v>190</v>
-      </c>
-      <c r="I31" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="J31" s="7">
-        <v>6</v>
-      </c>
-      <c r="K31" s="7"/>
+      <c r="E31" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="F31" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="G31" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="H31" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="I31" s="10" t="s">
+        <v>210</v>
+      </c>
+      <c r="J31" s="9">
+        <v>4</v>
+      </c>
+      <c r="K31" s="9"/>
     </row>
     <row r="32" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
@@ -2225,31 +2231,31 @@
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="C32" s="13" t="s">
+      <c r="C32" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="D32" s="9" t="s">
+      <c r="D32" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="E32" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="F32" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="G32" s="10" t="s">
-        <v>164</v>
-      </c>
-      <c r="H32" s="9" t="s">
-        <v>190</v>
-      </c>
-      <c r="I32" s="10" t="s">
-        <v>217</v>
-      </c>
-      <c r="J32" s="9">
-        <v>4</v>
-      </c>
-      <c r="K32" s="9"/>
+      <c r="E32" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="F32" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="G32" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="H32" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I32" s="8" t="s">
+        <v>211</v>
+      </c>
+      <c r="J32" s="7">
+        <v>1</v>
+      </c>
+      <c r="K32" s="7"/>
     </row>
     <row r="33" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
@@ -2257,31 +2263,31 @@
         <f>ROW(B33) - ROW($B$2)</f>
         <v>31</v>
       </c>
-      <c r="C33" s="12" t="s">
+      <c r="C33" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="D33" s="7" t="s">
+      <c r="D33" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="E33" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="F33" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="G33" s="8" t="s">
-        <v>165</v>
-      </c>
-      <c r="H33" s="7" t="s">
-        <v>190</v>
-      </c>
-      <c r="I33" s="8" t="s">
-        <v>218</v>
-      </c>
-      <c r="J33" s="7">
-        <v>1</v>
-      </c>
-      <c r="K33" s="7"/>
+      <c r="E33" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="F33" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="G33" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="H33" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="I33" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="J33" s="9">
+        <v>1</v>
+      </c>
+      <c r="K33" s="9"/>
     </row>
     <row r="34" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
@@ -2289,31 +2295,31 @@
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="C34" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="D34" s="9" t="s">
+      <c r="C34" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D34" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="E34" s="10" t="s">
-        <v>100</v>
-      </c>
-      <c r="F34" s="9" t="s">
-        <v>137</v>
-      </c>
-      <c r="G34" s="10" t="s">
-        <v>166</v>
-      </c>
-      <c r="H34" s="9" t="s">
-        <v>190</v>
-      </c>
-      <c r="I34" s="10" t="s">
-        <v>219</v>
-      </c>
-      <c r="J34" s="9">
-        <v>1</v>
-      </c>
-      <c r="K34" s="9"/>
+      <c r="E34" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="F34" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="G34" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="H34" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I34" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="J34" s="7">
+        <v>1</v>
+      </c>
+      <c r="K34" s="7"/>
     </row>
     <row r="35" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
@@ -2321,31 +2327,31 @@
         <f>ROW(B35) - ROW($B$2)</f>
         <v>33</v>
       </c>
-      <c r="C35" s="12" t="s">
+      <c r="C35" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="D35" s="7" t="s">
+      <c r="D35" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="E35" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="F35" s="7" t="s">
-        <v>135</v>
-      </c>
-      <c r="G35" s="8" t="s">
-        <v>167</v>
-      </c>
-      <c r="H35" s="7" t="s">
-        <v>190</v>
-      </c>
-      <c r="I35" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="J35" s="7">
-        <v>1</v>
-      </c>
-      <c r="K35" s="7"/>
+      <c r="E35" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="F35" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="G35" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="H35" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="I35" s="10" t="s">
+        <v>214</v>
+      </c>
+      <c r="J35" s="9">
+        <v>1</v>
+      </c>
+      <c r="K35" s="9"/>
     </row>
     <row r="36" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
@@ -2353,31 +2359,31 @@
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="C36" s="13" t="s">
+      <c r="C36" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="D36" s="9" t="s">
+      <c r="D36" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="E36" s="10" t="s">
-        <v>102</v>
-      </c>
-      <c r="F36" s="9" t="s">
-        <v>138</v>
-      </c>
-      <c r="G36" s="10" t="s">
-        <v>168</v>
-      </c>
-      <c r="H36" s="9" t="s">
-        <v>190</v>
-      </c>
-      <c r="I36" s="10" t="s">
-        <v>221</v>
-      </c>
-      <c r="J36" s="9">
-        <v>1</v>
-      </c>
-      <c r="K36" s="9"/>
+      <c r="E36" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="F36" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="G36" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="H36" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I36" s="8" t="s">
+        <v>215</v>
+      </c>
+      <c r="J36" s="7">
+        <v>1</v>
+      </c>
+      <c r="K36" s="7"/>
     </row>
     <row r="37" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
@@ -2385,31 +2391,31 @@
         <f>ROW(B37) - ROW($B$2)</f>
         <v>35</v>
       </c>
-      <c r="C37" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D37" s="7" t="s">
+      <c r="C37" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="D37" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="E37" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="F37" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="G37" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="H37" s="7" t="s">
-        <v>190</v>
-      </c>
-      <c r="I37" s="8" t="s">
-        <v>222</v>
-      </c>
-      <c r="J37" s="7">
-        <v>1</v>
-      </c>
-      <c r="K37" s="7"/>
+      <c r="E37" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="F37" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="G37" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="H37" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="I37" s="10" t="s">
+        <v>216</v>
+      </c>
+      <c r="J37" s="9">
+        <v>1</v>
+      </c>
+      <c r="K37" s="9"/>
     </row>
     <row r="38" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
@@ -2417,31 +2423,31 @@
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="C38" s="13" t="s">
+      <c r="C38" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="D38" s="9" t="s">
+      <c r="D38" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="E38" s="10" t="s">
-        <v>104</v>
-      </c>
-      <c r="F38" s="9" t="s">
-        <v>138</v>
-      </c>
-      <c r="G38" s="10" t="s">
-        <v>170</v>
-      </c>
-      <c r="H38" s="9" t="s">
-        <v>190</v>
-      </c>
-      <c r="I38" s="10" t="s">
-        <v>223</v>
-      </c>
-      <c r="J38" s="9">
-        <v>1</v>
-      </c>
-      <c r="K38" s="9"/>
+      <c r="E38" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="F38" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="G38" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="H38" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I38" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="J38" s="7">
+        <v>1</v>
+      </c>
+      <c r="K38" s="7"/>
     </row>
     <row r="39" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
@@ -2449,31 +2455,31 @@
         <f>ROW(B39) - ROW($B$2)</f>
         <v>37</v>
       </c>
-      <c r="C39" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="D39" s="7" t="s">
+      <c r="C39" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D39" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="E39" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="F39" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="G39" s="8" t="s">
-        <v>171</v>
-      </c>
-      <c r="H39" s="7" t="s">
-        <v>190</v>
-      </c>
-      <c r="I39" s="8" t="s">
-        <v>224</v>
-      </c>
-      <c r="J39" s="7">
-        <v>1</v>
-      </c>
-      <c r="K39" s="7"/>
+      <c r="E39" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="F39" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="G39" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="H39" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="I39" s="10" t="s">
+        <v>218</v>
+      </c>
+      <c r="J39" s="9">
+        <v>1</v>
+      </c>
+      <c r="K39" s="9"/>
     </row>
     <row r="40" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
@@ -2481,31 +2487,31 @@
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="C40" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="D40" s="9" t="s">
+      <c r="C40" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D40" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="E40" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="F40" s="9" t="s">
-        <v>138</v>
-      </c>
-      <c r="G40" s="10" t="s">
-        <v>172</v>
-      </c>
-      <c r="H40" s="9" t="s">
-        <v>190</v>
-      </c>
-      <c r="I40" s="10" t="s">
-        <v>225</v>
-      </c>
-      <c r="J40" s="9">
-        <v>1</v>
-      </c>
-      <c r="K40" s="9"/>
+      <c r="E40" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="F40" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="G40" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="H40" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I40" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="J40" s="7">
+        <v>1</v>
+      </c>
+      <c r="K40" s="7"/>
     </row>
     <row r="41" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
@@ -2513,31 +2519,31 @@
         <f>ROW(B41) - ROW($B$2)</f>
         <v>39</v>
       </c>
-      <c r="C41" s="12" t="s">
+      <c r="C41" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="D41" s="7" t="s">
+      <c r="D41" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="E41" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="F41" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="G41" s="8" t="s">
-        <v>173</v>
-      </c>
-      <c r="H41" s="7" t="s">
-        <v>190</v>
-      </c>
-      <c r="I41" s="8" t="s">
-        <v>226</v>
-      </c>
-      <c r="J41" s="7">
-        <v>1</v>
-      </c>
-      <c r="K41" s="7"/>
+      <c r="E41" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="F41" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="G41" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="H41" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="I41" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="J41" s="9">
+        <v>1</v>
+      </c>
+      <c r="K41" s="9"/>
     </row>
     <row r="42" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
@@ -2545,159 +2551,161 @@
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="C42" s="13" t="s">
+      <c r="C42" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="D42" s="9" t="s">
+      <c r="D42" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="E42" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="F42" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="G42" s="10" t="s">
-        <v>174</v>
-      </c>
-      <c r="H42" s="9" t="s">
-        <v>190</v>
-      </c>
-      <c r="I42" s="10" t="s">
-        <v>227</v>
-      </c>
-      <c r="J42" s="9">
-        <v>1</v>
-      </c>
-      <c r="K42" s="9"/>
-    </row>
-    <row r="43" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E42" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="F42" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="G42" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="H42" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I42" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="J42" s="7">
+        <v>1</v>
+      </c>
+      <c r="K42" s="7"/>
+    </row>
+    <row r="43" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="11">
         <f>ROW(B43) - ROW($B$2)</f>
         <v>41</v>
       </c>
-      <c r="C43" s="12" t="s">
+      <c r="C43" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="D43" s="7" t="s">
+      <c r="D43" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="E43" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="F43" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="G43" s="8" t="s">
-        <v>175</v>
-      </c>
-      <c r="H43" s="7" t="s">
-        <v>190</v>
-      </c>
-      <c r="I43" s="8" t="s">
-        <v>228</v>
-      </c>
-      <c r="J43" s="7">
-        <v>1</v>
-      </c>
-      <c r="K43" s="7"/>
-    </row>
-    <row r="44" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E43" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="F43" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="G43" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="H43" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="I43" s="10" t="s">
+        <v>222</v>
+      </c>
+      <c r="J43" s="9">
+        <v>12</v>
+      </c>
+      <c r="K43" s="9"/>
+    </row>
+    <row r="44" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
       <c r="B44" s="11">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="C44" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="D44" s="9" t="s">
+      <c r="C44" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D44" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="E44" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="F44" s="9" t="s">
-        <v>137</v>
-      </c>
-      <c r="G44" s="10" t="s">
-        <v>176</v>
-      </c>
-      <c r="H44" s="9" t="s">
-        <v>198</v>
-      </c>
-      <c r="I44" s="10" t="s">
-        <v>229</v>
-      </c>
-      <c r="J44" s="9">
-        <v>12</v>
-      </c>
-      <c r="K44" s="9"/>
-    </row>
-    <row r="45" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E44" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="F44" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="G44" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="H44" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="I44" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="J44" s="7">
+        <v>6</v>
+      </c>
+      <c r="K44" s="7"/>
+    </row>
+    <row r="45" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1"/>
       <c r="B45" s="11">
         <f>ROW(B45) - ROW($B$2)</f>
         <v>43</v>
       </c>
-      <c r="C45" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D45" s="7" t="s">
+      <c r="C45" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D45" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="E45" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="F45" s="7" t="s">
-        <v>137</v>
-      </c>
-      <c r="G45" s="8" t="s">
-        <v>177</v>
-      </c>
-      <c r="H45" s="7" t="s">
-        <v>190</v>
-      </c>
-      <c r="I45" s="8" t="s">
-        <v>225</v>
-      </c>
-      <c r="J45" s="7">
-        <v>6</v>
-      </c>
-      <c r="K45" s="7"/>
-    </row>
-    <row r="46" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E45" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="F45" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="G45" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="H45" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="I45" s="10" t="s">
+        <v>226</v>
+      </c>
+      <c r="J45" s="9">
+        <v>3</v>
+      </c>
+      <c r="K45" s="9"/>
+    </row>
+    <row r="46" spans="1:11" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
       <c r="B46" s="11">
         <f t="shared" si="0"/>
         <v>44</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>65</v>
+        <v>234</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>112</v>
+        <v>235</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="G46" s="10" t="s">
-        <v>140</v>
+        <v>236</v>
       </c>
       <c r="H46" s="9" t="s">
-        <v>190</v>
+        <v>226</v>
       </c>
       <c r="I46" s="10" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="J46" s="9">
-        <v>3</v>
-      </c>
-      <c r="K46" s="9"/>
+        <v>1</v>
+      </c>
+      <c r="K46" s="15" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="47" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1"/>
@@ -2709,22 +2717,22 @@
         <v>20</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="F47" s="7" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="H47" s="7" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="I47" s="10" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="J47" s="7">
         <v>1</v>
@@ -2741,22 +2749,22 @@
         <v>20</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E48" s="10" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="G48" s="10" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="H48" s="9" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="I48" s="10" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="J48" s="9">
         <v>1</v>
@@ -2773,22 +2781,22 @@
         <v>20</v>
       </c>
       <c r="D49" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E49" s="8" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="H49" s="7" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="I49" s="10" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="J49" s="7">
         <v>1</v>

</xml_diff>